<commit_message>
Callback de Peso para DN e MN
</commit_message>
<xml_diff>
--- a/Project_CNN/DenseNet/Resultados/Experimento 1 - DenseNet/training_metrics.xlsx
+++ b/Project_CNN/DenseNet/Resultados/Experimento 1 - DenseNet/training_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marci_wawp\Desktop\Arquivos\Mestrado\Projeto-Classificadores\Project_CNN\DenseNet\Resultados\Experimento 1 - DenseNet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7555C955-E742-4E64-AAA5-2572F46B3519}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{669BA485-90B4-4A80-8EA5-BE69E9D9E833}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5971,7 +5971,7 @@
       <xdr:rowOff>4762</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -6007,7 +6007,7 @@
       <xdr:rowOff>185736</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>46</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>

</xml_diff>